<commit_message>
Finalização das novas atualizações da Dalila
</commit_message>
<xml_diff>
--- a/exports/resultados_cnj.xlsx
+++ b/exports/resultados_cnj.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="89">
   <si>
     <t>Meta</t>
   </si>
@@ -166,9 +166,6 @@
     <t>Reduzir em 0,5 ponto percentual a taxa de congestionamento líquida de processo de conhecimento, em relação a 2024. Cláusula de barreira: 56%.</t>
   </si>
   <si>
-    <t>Total Meta 5</t>
-  </si>
-  <si>
     <t>83,53%</t>
   </si>
   <si>
@@ -184,9 +181,6 @@
     <t>Identificar e julgar até 31/12/2025 - 50% dos processos relacionados às ações ambientais distribuídos até 31/12/2024.</t>
   </si>
   <si>
-    <t>Total Meta 6</t>
-  </si>
-  <si>
     <t>90,88%</t>
   </si>
   <si>
@@ -272,9 +266,6 @@
   </si>
   <si>
     <t>Desenvolver, no ano de 2025, dois projetos relacionados à Agenda 2030 da ONU, oriundos do Laboratório de Inovação, com participação de pelo menos um laboratório de outra instituição pública, e que gerem benefícios à sociedade.</t>
-  </si>
-  <si>
-    <t>Total Meta 9</t>
   </si>
   <si>
     <t>Meta 10 – Promover os direitos da criança e do adolescente.</t>
@@ -307,7 +298,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -663,14 +654,14 @@
   <dimension ref="A1:E41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="3" width="77.86214285714286" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="3" width="47.29071428571429" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1035,10 +1026,10 @@
         <v>49</v>
       </c>
       <c r="C22" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>51</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>9</v>
@@ -1055,7 +1046,7 @@
         <v>10</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>9</v>
@@ -1072,7 +1063,7 @@
         <v>14</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>9</v>
@@ -1080,291 +1071,291 @@
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="C25" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="E25" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
       <c r="A27" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
       <c r="A28" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
       <c r="A29" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
       <c r="A30" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="D30" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="E30" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
       <c r="A31" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
       <c r="A32" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="D32" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>71</v>
-      </c>
       <c r="E32" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
       <c r="A33" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
       <c r="A35" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
       <c r="A36" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
       <c r="A37" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
       <c r="A38" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
       <c r="A39" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>86</v>
+        <v>16</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
       <c r="A40" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
       <c r="A41" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aplicações das alterações propostas pela Dalila 80% finalizadas
</commit_message>
<xml_diff>
--- a/exports/resultados_cnj.xlsx
+++ b/exports/resultados_cnj.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-04-28 12:17</t>
+          <t>2026-05-25 16:59</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-04-28 12:17</t>
+          <t>2026-05-25 16:59</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-04-28 12:17</t>
+          <t>2026-05-25 16:59</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-04-28 12:17</t>
+          <t>2026-05-25 16:59</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-04-28 12:17</t>
+          <t>2026-05-25 16:59</t>
         </is>
       </c>
     </row>
@@ -603,152 +603,152 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Processos mais Antigos</t>
+          <t>1º Grau</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>76,47%</t>
+          <t>107,66%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-04-28 12:18</t>
+          <t>2026-05-25 16:59</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Meta 3 – Estimular a conciliação</t>
+          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Aumentar o indicador Índice de Conciliação do Justiça em Números em 1 ponto percentual em relação a 2024. Cláusula de barreira: 17% de Índice de Conciliação.</t>
+          <t>Identificar e julgar até 31/12/2025 - pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>2º Grau</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>100,00%</t>
+          <t>108,23%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 16:59</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Meta 4 – Priorizar o julgamento dos processos relativos aos crimes contra a Administração Pública, à improbidade administrativa e aos ilícitos eleitorais</t>
+          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Identificar e julgar até 31/12/2025, 65% das ações de improbidade administrativa e das ações penais relacionadas a crimes contra a Administração Pública, distribuídas até 31/12/2021, em especial as relativas a corrupção ativa e passiva, peculato em geral e concussão e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021.</t>
+          <t>Identificar e julgar até 31/12/2025 - pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Total - Crimes Contra Adm.</t>
+          <t>Processos mais Antigos</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>143,66%</t>
+          <t>52,53%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 16:59</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Meta 4 – Priorizar o julgamento dos processos relativos aos crimes contra a Administração Pública, à improbidade administrativa e aos ilícitos eleitorais</t>
+          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Identificar e julgar até 31/12/2025, 65% das ações de improbidade administrativa e das ações penais relacionadas a crimes contra a Administração Pública, distribuídas até 31/12/2021, em especial as relativas a corrupção ativa e passiva, peculato em geral e concussão e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021.</t>
+          <t>Identificar e julgar até 31/12/2025 - pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Total - Improbidade</t>
+          <t>Juizado Especial</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>75,11%</t>
+          <t>99,64%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 16:59</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Meta 4 – Priorizar o julgamento dos processos relativos aos crimes contra a Administração Pública, à improbidade administrativa e aos ilícitos eleitorais</t>
+          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Identificar e julgar até 31/12/2025, 65% das ações de improbidade administrativa e das ações penais relacionadas a crimes contra a Administração Pública, distribuídas até 31/12/2021, em especial as relativas a corrupção ativa e passiva, peculato em geral e concussão e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021.</t>
+          <t>Identificar e julgar até 31/12/2025 - pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2º Grau - Crimes Contra Adm.</t>
+          <t>Turma Recursal</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>153,09%</t>
+          <t>100,97%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 16:59</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Meta 4 – Priorizar o julgamento dos processos relativos aos crimes contra a Administração Pública, à improbidade administrativa e aos ilícitos eleitorais</t>
+          <t>Meta 3 – Estimular a conciliação</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Identificar e julgar até 31/12/2025, 65% das ações de improbidade administrativa e das ações penais relacionadas a crimes contra a Administração Pública, distribuídas até 31/12/2021, em especial as relativas a corrupção ativa e passiva, peculato em geral e concussão e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021.</t>
+          <t>Aumentar o indicador Índice de Conciliação do Justiça em Números em 1 ponto percentual em relação a 2024. Cláusula de barreira: 17% de Índice de Conciliação.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Juizado Especial - Crimes Contra Adm.</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>149,07%</t>
+          <t>100,00%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
@@ -765,17 +765,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Turma Recursal - Crimes Contra Adm.</t>
+          <t>Total - Crimes Contra Adm.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>147,37%</t>
+          <t>143,66%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
@@ -792,17 +792,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1º Grau - Crimes Contra Adm.</t>
+          <t>Total - Improbidade</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>136,63%</t>
+          <t>75,11%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
@@ -819,17 +819,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2º Grau - Improbidade</t>
+          <t>2º Grau - Crimes Contra Adm.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>98,69%</t>
+          <t>153,09%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
@@ -846,17 +846,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Juizado Especial - Improbidade</t>
+          <t>Juizado Especial - Crimes Contra Adm.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>66,67%</t>
+          <t>149,07%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
@@ -873,395 +873,395 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1º Grau - Improbidade</t>
+          <t>Turma Recursal - Crimes Contra Adm.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>70,79%</t>
+          <t>147,37%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Meta 5 – Reduzir a taxa de congestionamento</t>
+          <t>Meta 4 – Priorizar o julgamento dos processos relativos aos crimes contra a Administração Pública, à improbidade administrativa e aos ilícitos eleitorais</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Reduzir em 0,5 ponto percentual a taxa de congestionamento líquida de processo de conhecimento, em relação a 2024. Cláusula de barreira: 56%.</t>
+          <t>Identificar e julgar até 31/12/2025, 65% das ações de improbidade administrativa e das ações penais relacionadas a crimes contra a Administração Pública, distribuídas até 31/12/2021, em especial as relativas a corrupção ativa e passiva, peculato em geral e concussão e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Total Meta 5</t>
+          <t>1º Grau - Crimes Contra Adm.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>85,78%</t>
+          <t>136,63%</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Meta 5 – Reduzir a taxa de congestionamento</t>
+          <t>Meta 4 – Priorizar o julgamento dos processos relativos aos crimes contra a Administração Pública, à improbidade administrativa e aos ilícitos eleitorais</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Reduzir em 0,5 ponto percentual a taxa de congestionamento líquida de processo de conhecimento, em relação a 2024. Cláusula de barreira: 56%.</t>
+          <t>Identificar e julgar até 31/12/2025, 65% das ações de improbidade administrativa e das ações penais relacionadas a crimes contra a Administração Pública, distribuídas até 31/12/2021, em especial as relativas a corrupção ativa e passiva, peculato em geral e concussão e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1º Grau</t>
+          <t>2º Grau - Improbidade</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>108,34%</t>
+          <t>98,69%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Meta 6 – Priorizar o julgamento das ações ambientais</t>
+          <t>Meta 4 – Priorizar o julgamento dos processos relativos aos crimes contra a Administração Pública, à improbidade administrativa e aos ilícitos eleitorais</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Identificar e julgar até 31/12/2025 - 50% dos processos relacionados às ações ambientais distribuídos até 31/12/2024.</t>
+          <t>Identificar e julgar até 31/12/2025, 65% das ações de improbidade administrativa e das ações penais relacionadas a crimes contra a Administração Pública, distribuídas até 31/12/2021, em especial as relativas a corrupção ativa e passiva, peculato em geral e concussão e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Total Meta 6</t>
+          <t>Juizado Especial - Improbidade</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>94,02%</t>
+          <t>66,67%</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Meta 6 – Priorizar o julgamento das ações ambientais</t>
+          <t>Meta 4 – Priorizar o julgamento dos processos relativos aos crimes contra a Administração Pública, à improbidade administrativa e aos ilícitos eleitorais</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Identificar e julgar até 31/12/2025 - 50% dos processos relacionados às ações ambientais distribuídos até 31/12/2024.</t>
+          <t>Identificar e julgar até 31/12/2025, 65% das ações de improbidade administrativa e das ações penais relacionadas a crimes contra a Administração Pública, distribuídas até 31/12/2021, em especial as relativas a corrupção ativa e passiva, peculato em geral e concussão e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Turma Recursal</t>
+          <t>1º Grau - Improbidade</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>176,27%</t>
+          <t>70,79%</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Meta 6 – Priorizar o julgamento das ações ambientais</t>
+          <t>Meta 5 – Reduzir a taxa de congestionamento</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Identificar e julgar até 31/12/2025 - 50% dos processos relacionados às ações ambientais distribuídos até 31/12/2024.</t>
+          <t>Reduzir em 0,5 ponto percentual a taxa de congestionamento líquida de processo de conhecimento, em relação a 2024. Cláusula de barreira: 56%.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2º Grau</t>
+          <t>Total Meta 5</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>165,85%</t>
+          <t>85,78%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Meta 6 – Priorizar o julgamento das ações ambientais</t>
+          <t>Meta 5 – Reduzir a taxa de congestionamento</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Identificar e julgar até 31/12/2025 - 50% dos processos relacionados às ações ambientais distribuídos até 31/12/2024.</t>
+          <t>Reduzir em 0,5 ponto percentual a taxa de congestionamento líquida de processo de conhecimento, em relação a 2024. Cláusula de barreira: 56%.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Juizado Especial</t>
+          <t>1º Grau</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>152,62%</t>
+          <t>90,34%</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Meta 6 – Priorizar o julgamento das ações ambientais</t>
+          <t>Meta 5 – Reduzir a taxa de congestionamento</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Identificar e julgar até 31/12/2025 - 50% dos processos relacionados às ações ambientais distribuídos até 31/12/2024.</t>
+          <t>Reduzir em 0,5 ponto percentual a taxa de congestionamento líquida de processo de conhecimento, em relação a 2024. Cláusula de barreira: 56%.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1º Grau</t>
+          <t>Juizado Especial</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>144,87%</t>
+          <t>73,80%</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-04-28 12:19</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Meta 7 – Priorizar o julgamento dos processos relacionados aos indígenas e quilombolas</t>
+          <t>Meta 6 – Priorizar o julgamento das ações ambientais</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Identificar e julgar até 31/12/2025 - 50% dos processos relacionados aos direitos das comunidades indígenas e 50% dos processos relacionados aos direitos das comunidades quilombolas distribuídos até 31/12/2024.</t>
+          <t>Identificar e julgar até 31/12/2025 - 50% dos processos relacionados às ações ambientais distribuídos até 31/12/2024.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Total Indígenas</t>
+          <t>Total Meta 6</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>120,00%</t>
+          <t>94,02%</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-04-28 12:20</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Meta 7 – Priorizar o julgamento dos processos relacionados aos indígenas e quilombolas</t>
+          <t>Meta 6 – Priorizar o julgamento das ações ambientais</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Identificar e julgar até 31/12/2025 - 50% dos processos relacionados aos direitos das comunidades indígenas e 50% dos processos relacionados aos direitos das comunidades quilombolas distribuídos até 31/12/2024.</t>
+          <t>Identificar e julgar até 31/12/2025 - 50% dos processos relacionados às ações ambientais distribuídos até 31/12/2024.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Total Quilombola</t>
+          <t>Turma Recursal</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>100,00%</t>
+          <t>180,43%</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-04-28 12:20</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Meta 8 – Priorizar o julgamento dos processos relacionados ao feminicídio e à violência doméstica e familiar contra as mulheres</t>
+          <t>Meta 6 – Priorizar o julgamento das ações ambientais</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Identificar e julgar, até 31/12/2025 - 75% dos casos de feminicídio distribuídos até 31/12/2023 e 90% dos casos de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023.</t>
+          <t>Identificar e julgar até 31/12/2025 - 50% dos processos relacionados às ações ambientais distribuídos até 31/12/2024.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Total Violência Doméstica</t>
+          <t>2º Grau</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>93,12%</t>
+          <t>141,62%</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-04-28 12:20</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Meta 8 – Priorizar o julgamento dos processos relacionados ao feminicídio e à violência doméstica e familiar contra as mulheres</t>
+          <t>Meta 6 – Priorizar o julgamento das ações ambientais</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Identificar e julgar, até 31/12/2025 - 75% dos casos de feminicídio distribuídos até 31/12/2023 e 90% dos casos de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023.</t>
+          <t>Identificar e julgar até 31/12/2025 - 50% dos processos relacionados às ações ambientais distribuídos até 31/12/2024.</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Total Feminicídio</t>
+          <t>Juizado Especial</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>112,56%</t>
+          <t>109,55%</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-04-28 12:20</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Meta 8 – Priorizar o julgamento dos processos relacionados ao feminicídio e à violência doméstica e familiar contra as mulheres</t>
+          <t>Meta 6 – Priorizar o julgamento das ações ambientais</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Identificar e julgar, até 31/12/2025 - 75% dos casos de feminicídio distribuídos até 31/12/2023 e 90% dos casos de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023.</t>
+          <t>Identificar e julgar até 31/12/2025 - 50% dos processos relacionados às ações ambientais distribuídos até 31/12/2024.</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2º Grau - Violência Doméstica</t>
+          <t>1º Grau</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>100,48%</t>
+          <t>67,48%</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-04-28 12:20</t>
+          <t>2026-05-25 17:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Meta 8 – Priorizar o julgamento dos processos relacionados ao feminicídio e à violência doméstica e familiar contra as mulheres</t>
+          <t>Meta 7 – Priorizar o julgamento dos processos relacionados aos indígenas e quilombolas</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Identificar e julgar, até 31/12/2025 - 75% dos casos de feminicídio distribuídos até 31/12/2023 e 90% dos casos de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023.</t>
+          <t>Identificar e julgar até 31/12/2025 - 50% dos processos relacionados aos direitos das comunidades indígenas e 50% dos processos relacionados aos direitos das comunidades quilombolas distribuídos até 31/12/2024.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1º Grau - Violência Doméstica</t>
+          <t>Total Indígenas</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>92,79%</t>
+          <t>120,00%</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-04-28 12:20</t>
+          <t>2026-05-25 17:01</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Meta 8 – Priorizar o julgamento dos processos relacionados ao feminicídio e à violência doméstica e familiar contra as mulheres</t>
+          <t>Meta 7 – Priorizar o julgamento dos processos relacionados aos indígenas e quilombolas</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Identificar e julgar, até 31/12/2025 - 75% dos casos de feminicídio distribuídos até 31/12/2023 e 90% dos casos de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023.</t>
+          <t>Identificar e julgar até 31/12/2025 - 50% dos processos relacionados aos direitos das comunidades indígenas e 50% dos processos relacionados aos direitos das comunidades quilombolas distribuídos até 31/12/2024.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Juizado Especial - Violência Doméstica</t>
+          <t>Total Quilombola</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>82,49%</t>
+          <t>100,00%</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-04-28 12:20</t>
+          <t>2026-05-25 17:01</t>
         </is>
       </c>
     </row>
@@ -1278,17 +1278,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2º Grau - Feminicídio</t>
+          <t>Total Violência Doméstica</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>128,89%</t>
+          <t>93,12%</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-04-28 12:20</t>
+          <t>2026-05-25 17:01</t>
         </is>
       </c>
     </row>
@@ -1305,98 +1305,233 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1º Grau - Feminicídio</t>
+          <t>Total Feminicídio</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>103,25%</t>
+          <t>112,56%</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-04-28 12:20</t>
+          <t>2026-05-25 17:01</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Meta 9 – Estimular a inovação no Poder Judiciário</t>
+          <t>Meta 8 – Priorizar o julgamento dos processos relacionados ao feminicídio e à violência doméstica e familiar contra as mulheres</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Desenvolver, no ano de 2025, dois projetos relacionados à Agenda 2030 da ONU, oriundos do Laboratório de Inovação, com participação de pelo menos um laboratório de outra instituição pública, e que gerem benefícios à sociedade.</t>
+          <t>Identificar e julgar, até 31/12/2025 - 75% dos casos de feminicídio distribuídos até 31/12/2023 e 90% dos casos de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023.</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Total Meta 9</t>
+          <t>2º Grau - Violência Doméstica</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>100,00%</t>
+          <t>100,48%</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-04-28 12:20</t>
+          <t>2026-05-25 17:01</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Meta 10 – Promover os direitos da criança e do adolescente.</t>
+          <t>Meta 8 – Priorizar o julgamento dos processos relacionados ao feminicídio e à violência doméstica e familiar contra as mulheres</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Identificar e julgar, até 31/12/2025, no 1º grau, 90% e no 2º grau, 100% dos processos em fase de conhecimento, nas competências da Infância e Juventude cível e de apuração de ato infracional, distribuídos até 31/12/2023 nas respectivas instâncias.</t>
+          <t>Identificar e julgar, até 31/12/2025 - 75% dos casos de feminicídio distribuídos até 31/12/2023 e 90% dos casos de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>1º Grau</t>
+          <t>1º Grau - Violência Doméstica</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>88,84%</t>
+          <t>92,79%</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-04-28 12:20</t>
+          <t>2026-05-25 17:01</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>Meta 8 – Priorizar o julgamento dos processos relacionados ao feminicídio e à violência doméstica e familiar contra as mulheres</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Identificar e julgar, até 31/12/2025 - 75% dos casos de feminicídio distribuídos até 31/12/2023 e 90% dos casos de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023.</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Juizado Especial - Violência Doméstica</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>82,49%</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-05-25 17:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Meta 8 – Priorizar o julgamento dos processos relacionados ao feminicídio e à violência doméstica e familiar contra as mulheres</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Identificar e julgar, até 31/12/2025 - 75% dos casos de feminicídio distribuídos até 31/12/2023 e 90% dos casos de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023.</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2º Grau - Feminicídio</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>128,89%</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-05-25 17:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Meta 8 – Priorizar o julgamento dos processos relacionados ao feminicídio e à violência doméstica e familiar contra as mulheres</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Identificar e julgar, até 31/12/2025 - 75% dos casos de feminicídio distribuídos até 31/12/2023 e 90% dos casos de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023.</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1º Grau - Feminicídio</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>103,25%</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-05-25 17:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Meta 9 – Estimular a inovação no Poder Judiciário</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Desenvolver, no ano de 2025, dois projetos relacionados à Agenda 2030 da ONU, oriundos do Laboratório de Inovação, com participação de pelo menos um laboratório de outra instituição pública, e que gerem benefícios à sociedade.</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Total Meta 9</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2026-05-25 17:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>Meta 10 – Promover os direitos da criança e do adolescente.</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>Identificar e julgar, até 31/12/2025, no 1º grau, 90% e no 2º grau, 100% dos processos em fase de conhecimento, nas competências da Infância e Juventude cível e de apuração de ato infracional, distribuídos até 31/12/2023 nas respectivas instâncias.</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1º Grau</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>88,84%</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-05-25 17:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Meta 10 – Promover os direitos da criança e do adolescente.</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Identificar e julgar, até 31/12/2025, no 1º grau, 90% e no 2º grau, 100% dos processos em fase de conhecimento, nas competências da Infância e Juventude cível e de apuração de ato infracional, distribuídos até 31/12/2023 nas respectivas instâncias.</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
         <is>
           <t>2º Grau</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>85,03%</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>2026-04-28 12:20</t>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-05-25 17:01</t>
         </is>
       </c>
     </row>

</xml_diff>